<commit_message>
First implementation Rth/Cth Matrix
1) Implementation
2) Adding data
</commit_message>
<xml_diff>
--- a/config/default/default.xlsx
+++ b/config/default/default.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\q516645\Desktop\Github_ext\TherMOS\config\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4F52FCA0-B855-49F1-9A34-069EE2632F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB913290-8124-44AB-A8FB-BDA6D1543034}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0953EA25-A225-4AF7-A5B3-27A5BB5D0B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-18120" yWindow="-2550" windowWidth="18240" windowHeight="28440" activeTab="3" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="2" r:id="rId1"/>
@@ -1457,7 +1457,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1473,9 +1473,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1513,7 +1513,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1619,7 +1619,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1770,7 +1770,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA655AC4-52E1-45C0-83AC-CC64B56C05A9}">
   <dimension ref="A1:L18"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1930,7 +1930,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CAB857B-5D2E-4BE1-B462-B4B5EEAA4370}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>
@@ -1978,7 +1978,7 @@
         <v>107</v>
       </c>
       <c r="F2" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="29" t="s">
         <v>16</v>
@@ -2332,7 +2332,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86190CFD-1D2B-4FE4-A04E-A3C453840C86}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" customWidth="1"/>
@@ -2736,7 +2736,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799FBFCB-8244-4B83-8CC9-EBD2890613E5}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>
@@ -3958,7 +3958,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245B3F0A-B85A-4162-A12D-AC7176B54015}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>
@@ -4410,4 +4410,10 @@
     <oddFooter>&amp;C_x000D_&amp;1#&amp;"BMW Group Condensed"&amp;12&amp;KC00000 CONFIDENTIAL</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{e6935750-240b-48e4-a615-66942a738439}" enabled="1" method="Standard" siteId="{ce849bab-cc1c-465b-b62e-18f07c9ac198}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Adding SF to main
</commit_message>
<xml_diff>
--- a/config/default/default.xlsx
+++ b/config/default/default.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\q516645\Desktop\Github_ext\TherMOS\config\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/TherMOS/config/default/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0953EA25-A225-4AF7-A5B3-27A5BB5D0B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{0953EA25-A225-4AF7-A5B3-27A5BB5D0B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0137DD51-CFEF-4C7A-AFC2-58ACD8949FED}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{DB7D2548-4471-4992-93B1-3EC0BA66F7EA}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="2" r:id="rId1"/>
@@ -1457,7 +1457,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1473,9 +1473,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1513,7 +1513,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1619,7 +1619,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1770,7 +1770,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA655AC4-52E1-45C0-83AC-CC64B56C05A9}">
   <dimension ref="A1:L18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="18.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1930,7 +1930,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CAB857B-5D2E-4BE1-B462-B4B5EEAA4370}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>
@@ -1978,7 +1978,7 @@
         <v>107</v>
       </c>
       <c r="F2" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G2" s="29" t="s">
         <v>16</v>
@@ -2332,7 +2332,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86190CFD-1D2B-4FE4-A04E-A3C453840C86}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" customWidth="1"/>
@@ -2736,7 +2736,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{799FBFCB-8244-4B83-8CC9-EBD2890613E5}">
   <dimension ref="A1:G53"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="29.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>
@@ -3958,7 +3958,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245B3F0A-B85A-4162-A12D-AC7176B54015}">
   <dimension ref="A1:G26"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.109375" style="37" customWidth="1"/>

</xml_diff>